<commit_message>
add V_cap and M_cap columns to piles sheet, fix column letters and docs
- Add V_cap (shear capacity) and M_cap (moment capacity) columns N and O
  to the piles input template for future structural capacity checks
- Fix column letters in documentation to match actual sheet layout
  (A=# row number, so all fields shifted by one)
- Categorize columns as LEM only, FEM only, or LEM & FEM
- Clarify that S is needed beyond Ito & Matsui (capacity checks,
  per-pile force reporting)
- Move capacity checks plan from plan_piles_examples.md to plan_piles.md
  Section 9, covering both LEM (cap F_pile before converting to H) and
  FEM (elastic-perfectly-plastic via viscoplastic corrections)
- Use V_cap/M_cap notation consistently

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/inputs/input_template_v10.xlsx
+++ b/docs/inputs/input_template_v10.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33D3DEEB-13E6-6644-AAE3-D3DC72101951}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BBAABD4-E426-8F49-8470-E5780033835C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11520" yWindow="3160" windowWidth="27840" windowHeight="20620" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="24480" yWindow="2380" windowWidth="42700" windowHeight="22800" activeTab="11" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="180">
   <si>
     <t>X</t>
   </si>
@@ -696,15 +696,9 @@
     <t>Polygon #15</t>
   </si>
   <si>
-    <t>label</t>
-  </si>
-  <si>
     <t>H</t>
   </si>
   <si>
-    <t>theta</t>
-  </si>
-  <si>
     <t>D</t>
   </si>
   <si>
@@ -714,20 +708,54 @@
     <t>I</t>
   </si>
   <si>
-    <t>Required for LEM only</t>
-  </si>
-  <si>
-    <t>Optional</t>
-  </si>
-  <si>
     <t xml:space="preserve">Polygons coordinates can be input in CW or CCW order. </t>
+  </si>
+  <si>
+    <t>Vcap</t>
+  </si>
+  <si>
+    <t>Mcap</t>
+  </si>
+  <si>
+    <t>Label</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="0"/>
+        <rFont val="Symbol"/>
+        <charset val="2"/>
+      </rPr>
+      <t>q</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="0"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>p</t>
+    </r>
+  </si>
+  <si>
+    <t>LEM only</t>
+  </si>
+  <si>
+    <t>LEM &amp; FEM</t>
+  </si>
+  <si>
+    <t>FEM only</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -850,6 +878,13 @@
       <sz val="12"/>
       <color theme="0"/>
       <name val="Aptos Narrow (Body)"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="0"/>
+      <name val="Symbol"/>
+      <charset val="2"/>
     </font>
   </fonts>
   <fills count="17">
@@ -1036,7 +1071,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1158,9 +1193,6 @@
     <xf numFmtId="0" fontId="16" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1168,13 +1200,13 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1200,6 +1232,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -8246,6 +8284,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000039-9273-8E45-8E0C-DF8E6C08CDD2}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:xVal>
             <c:numRef>
@@ -8391,668 +8434,6 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000050-A2F6-274C-9E15-3D60CC318540}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="87"/>
-          <c:order val="87"/>
-          <c:tx>
-            <c:v>Pile #11</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent4">
-                    <a:lumMod val="50000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-          </c:marker>
-          <c:dPt>
-            <c:idx val="0"/>
-            <c:marker>
-              <c:symbol val="circle"/>
-              <c:size val="5"/>
-              <c:spPr>
-                <a:solidFill>
-                  <a:schemeClr val="accent4">
-                    <a:lumMod val="50000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:ln w="9525">
-                  <a:solidFill>
-                    <a:schemeClr val="accent4">
-                      <a:lumMod val="50000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                </a:ln>
-                <a:effectLst/>
-              </c:spPr>
-            </c:marker>
-            <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:ln w="19050" cap="rnd">
-                <a:solidFill>
-                  <a:schemeClr val="accent4">
-                    <a:lumMod val="50000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:round/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-          </c:dPt>
-          <c:xVal>
-            <c:numRef>
-              <c:f>(piles!$C$13,piles!$E$13)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>(piles!$D$13,piles!$F$13)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000051-A2F6-274C-9E15-3D60CC318540}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="88"/>
-          <c:order val="88"/>
-          <c:tx>
-            <c:v>Pile #12</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent5">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent5">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent5">
-                    <a:lumMod val="50000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>(piles!$C$14,piles!$E$14)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>(piles!$D$14,piles!$F$14)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000052-A2F6-274C-9E15-3D60CC318540}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="89"/>
-          <c:order val="89"/>
-          <c:tx>
-            <c:v>Pile #13</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent6">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent6">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent6">
-                    <a:lumMod val="50000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>(piles!$C$15,piles!$E$15)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>(piles!$D$15,piles!$F$15)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000053-A2F6-274C-9E15-3D60CC318540}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="90"/>
-          <c:order val="90"/>
-          <c:tx>
-            <c:v>Pile #14</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent1">
-                  <a:lumMod val="70000"/>
-                  <a:lumOff val="30000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent1">
-                  <a:lumMod val="70000"/>
-                  <a:lumOff val="30000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent1">
-                    <a:lumMod val="70000"/>
-                    <a:lumOff val="30000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>(piles!$C$16,piles!$E$16)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>(piles!$D$16,piles!$F$16)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000054-A2F6-274C-9E15-3D60CC318540}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="91"/>
-          <c:order val="91"/>
-          <c:tx>
-            <c:v>Pile #15</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent2">
-                  <a:lumMod val="70000"/>
-                  <a:lumOff val="30000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent2">
-                  <a:lumMod val="70000"/>
-                  <a:lumOff val="30000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent2">
-                    <a:lumMod val="70000"/>
-                    <a:lumOff val="30000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>(piles!$C$17,piles!$E$17)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>(piles!$D$17,piles!$F$17)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000055-A2F6-274C-9E15-3D60CC318540}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="92"/>
-          <c:order val="92"/>
-          <c:tx>
-            <c:v>Pile #16</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent3">
-                  <a:lumMod val="70000"/>
-                  <a:lumOff val="30000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent3">
-                  <a:lumMod val="70000"/>
-                  <a:lumOff val="30000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent3">
-                    <a:lumMod val="70000"/>
-                    <a:lumOff val="30000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>(piles!$C$18,piles!$E$18)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>(piles!$D$18,piles!$F$18)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000056-A2F6-274C-9E15-3D60CC318540}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="93"/>
-          <c:order val="93"/>
-          <c:tx>
-            <c:v>Pile #17</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="70000"/>
-                  <a:lumOff val="30000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="70000"/>
-                  <a:lumOff val="30000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent4">
-                    <a:lumMod val="70000"/>
-                    <a:lumOff val="30000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>(piles!$C$19,piles!$E$19)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>(piles!$D$19,piles!$F$19)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000057-A2F6-274C-9E15-3D60CC318540}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="94"/>
-          <c:order val="94"/>
-          <c:tx>
-            <c:v>Pile #18</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent5">
-                  <a:lumMod val="70000"/>
-                  <a:lumOff val="30000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent5">
-                  <a:lumMod val="70000"/>
-                  <a:lumOff val="30000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent5">
-                    <a:lumMod val="70000"/>
-                    <a:lumOff val="30000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>(piles!$C$20,piles!$E$20)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>(piles!$D$20,piles!$F$20)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000058-A2F6-274C-9E15-3D60CC318540}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="95"/>
-          <c:order val="95"/>
-          <c:tx>
-            <c:v>Pile #19</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent6">
-                  <a:lumMod val="70000"/>
-                  <a:lumOff val="30000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent6">
-                  <a:lumMod val="70000"/>
-                  <a:lumOff val="30000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent6">
-                    <a:lumMod val="70000"/>
-                    <a:lumOff val="30000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>(piles!$C$21,piles!$E$21)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>(piles!$D$21,piles!$F$21)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000059-A2F6-274C-9E15-3D60CC318540}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="96"/>
-          <c:order val="96"/>
-          <c:tx>
-            <c:v>Pile #20</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent1">
-                  <a:lumMod val="70000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent1">
-                  <a:lumMod val="70000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent1">
-                    <a:lumMod val="70000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>(piles!$C$22,piles!$E$22)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>(piles!$D$22,piles!$F$22)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{0000005A-A2F6-274C-9E15-3D60CC318540}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -10064,16 +9445,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>553357</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>99787</xdr:rowOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>290285</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>18144</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>426357</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>54428</xdr:rowOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>163285</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -10088,8 +9469,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="10885714" y="498930"/>
-          <a:ext cx="4826000" cy="2748641"/>
+          <a:off x="12273642" y="217715"/>
+          <a:ext cx="4826000" cy="1841499"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -10137,9 +9518,6 @@
           </a:r>
         </a:p>
         <a:p>
-          <a:endParaRPr lang="en-US" sz="1100" baseline="0"/>
-        </a:p>
-        <a:p>
           <a:r>
             <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
             <a:t>H</a:t>
@@ -10150,12 +9528,15 @@
           </a:r>
         </a:p>
         <a:p>
-          <a:endParaRPr lang="en-US" sz="1100" baseline="0"/>
-        </a:p>
-        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0">
+              <a:latin typeface="Symbol" pitchFamily="2" charset="2"/>
+            </a:rPr>
+            <a:t>q</a:t>
+          </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
-            <a:t>theta</a:t>
+            <a:t>p</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1100" baseline="0"/>
@@ -10171,11 +9552,8 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>Force angle from horizontal in degrees (default 0°; positive = upward)</a:t>
+            <a:t>Force angle from horizontal in degrees (degrees)</a:t>
           </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1100" baseline="0"/>
         </a:p>
         <a:p>
           <a:r>
@@ -10196,11 +9574,29 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>Pile diameter.</a:t>
+            <a:t>Pile diameter</a:t>
           </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1100" baseline="0"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> (ft or m)</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0">
+            <a:solidFill>
+              <a:schemeClr val="dk1"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+          </a:endParaRPr>
         </a:p>
         <a:p>
           <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
@@ -10230,11 +9626,8 @@
           </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1100" baseline="0"/>
-            <a:t>.</a:t>
+            <a:t> (ft or m)</a:t>
           </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1100" baseline="0"/>
         </a:p>
         <a:p>
           <a:r>
@@ -10243,11 +9636,8 @@
           </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1100" baseline="0"/>
-            <a:t> = Young's modulus of pile material</a:t>
+            <a:t> = Young's modulus of pile material (force/lengh^2)</a:t>
           </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1100" baseline="0"/>
         </a:p>
         <a:p>
           <a:r>
@@ -10268,43 +9658,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>Moment of inertia (computed from</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" b="0" i="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t> D</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="ar-AE" sz="1100" b="0" i="0">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t> </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" b="0" i="0">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>if omitted)</a:t>
+            <a:t>Moment of inertia (length^4)</a:t>
           </a:r>
           <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" baseline="0">
             <a:solidFill>
@@ -10317,9 +9671,6 @@
           </a:endParaRPr>
         </a:p>
         <a:p>
-          <a:endParaRPr lang="en-US" sz="1100" baseline="0"/>
-        </a:p>
-        <a:p>
           <a:r>
             <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
             <a:t>Area</a:t>
@@ -10338,10 +9689,12 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>Cross-sectional area (computed from</a:t>
+            <a:t>Cross-sectional area (length^2)</a:t>
           </a:r>
+        </a:p>
+        <a:p>
           <a:r>
-            <a:rPr lang="en-US" sz="1100" b="0" i="0" baseline="0">
+            <a:rPr lang="en-US" sz="1100" b="1" i="0">
               <a:solidFill>
                 <a:schemeClr val="dk1"/>
               </a:solidFill>
@@ -10350,10 +9703,10 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t> D</a:t>
+            <a:t>Vcap</a:t>
           </a:r>
           <a:r>
-            <a:rPr lang="ar-AE" sz="1100" b="0" i="0">
+            <a:rPr lang="en-US" sz="1100" b="0" i="0">
               <a:solidFill>
                 <a:schemeClr val="dk1"/>
               </a:solidFill>
@@ -10362,10 +9715,10 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t> </a:t>
+            <a:t> = Shear</a:t>
           </a:r>
           <a:r>
-            <a:rPr lang="en-US" sz="1100" b="0" i="0">
+            <a:rPr lang="en-US" sz="1100" b="0" i="0" baseline="0">
               <a:solidFill>
                 <a:schemeClr val="dk1"/>
               </a:solidFill>
@@ -10374,7 +9727,33 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>if omitted)</a:t>
+            <a:t> capacity of pile (force)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Mcap</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> = Moment capacity of pile (force x length)</a:t>
           </a:r>
           <a:endParaRPr lang="en-US" sz="1100"/>
         </a:p>
@@ -10731,11 +10110,11 @@
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B7" s="47" t="s">
+      <c r="B7" s="46" t="s">
         <v>47</v>
       </c>
-      <c r="C7" s="47"/>
-      <c r="D7" s="47"/>
+      <c r="C7" s="46"/>
+      <c r="D7" s="46"/>
       <c r="F7" s="15" t="s">
         <v>15</v>
       </c>
@@ -10894,36 +10273,36 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B2" s="57" t="s">
+      <c r="B2" s="56" t="s">
         <v>145</v>
       </c>
-      <c r="C2" s="57"/>
-      <c r="D2" s="57"/>
-      <c r="F2" s="57" t="s">
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="F2" s="56" t="s">
         <v>146</v>
       </c>
-      <c r="G2" s="57"/>
-      <c r="H2" s="57"/>
-      <c r="J2" s="57" t="s">
+      <c r="G2" s="56"/>
+      <c r="H2" s="56"/>
+      <c r="J2" s="56" t="s">
         <v>147</v>
       </c>
-      <c r="K2" s="57"/>
-      <c r="L2" s="57"/>
-      <c r="N2" s="57" t="s">
+      <c r="K2" s="56"/>
+      <c r="L2" s="56"/>
+      <c r="N2" s="56" t="s">
         <v>148</v>
       </c>
-      <c r="O2" s="57"/>
-      <c r="P2" s="57"/>
-      <c r="R2" s="57" t="s">
+      <c r="O2" s="56"/>
+      <c r="P2" s="56"/>
+      <c r="R2" s="56" t="s">
         <v>149</v>
       </c>
-      <c r="S2" s="57"/>
-      <c r="T2" s="57"/>
-      <c r="V2" s="57" t="s">
+      <c r="S2" s="56"/>
+      <c r="T2" s="56"/>
+      <c r="V2" s="56" t="s">
         <v>150</v>
       </c>
-      <c r="W2" s="57"/>
-      <c r="X2" s="57"/>
+      <c r="W2" s="56"/>
+      <c r="X2" s="56"/>
     </row>
     <row r="3" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">
@@ -11742,20 +11121,21 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C542BD7-5686-4248-AC02-D49DB39A8FC0}">
-  <dimension ref="A2:P25"/>
+  <dimension ref="A2:R15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4.83203125" style="1" customWidth="1"/>
     <col min="2" max="2" width="11.5" style="1" customWidth="1"/>
-    <col min="3" max="13" width="10.83203125" style="1"/>
+    <col min="3" max="15" width="10.83203125" style="1"/>
+    <col min="16" max="16" width="3.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
         <v>25</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="C2" s="12" t="s">
         <v>103</v>
@@ -11769,29 +11149,35 @@
       <c r="F2" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="G2" s="45" t="s">
+      <c r="G2" s="59" t="s">
+        <v>168</v>
+      </c>
+      <c r="H2" s="59" t="s">
+        <v>176</v>
+      </c>
+      <c r="I2" s="32" t="s">
         <v>169</v>
       </c>
-      <c r="H2" s="32" t="s">
+      <c r="J2" s="32" t="s">
         <v>170</v>
-      </c>
-      <c r="I2" s="32" t="s">
-        <v>171</v>
-      </c>
-      <c r="J2" s="32" t="s">
-        <v>172</v>
       </c>
       <c r="K2" s="33" t="s">
         <v>101</v>
       </c>
       <c r="L2" s="33" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="M2" s="33" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N2" s="60" t="s">
+        <v>173</v>
+      </c>
+      <c r="O2" s="60" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>1</v>
       </c>
@@ -11807,8 +11193,10 @@
       <c r="K3" s="3"/>
       <c r="L3" s="3"/>
       <c r="M3" s="3"/>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N3" s="3"/>
+      <c r="O3" s="3"/>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>2</v>
       </c>
@@ -11824,8 +11212,10 @@
       <c r="K4" s="3"/>
       <c r="L4" s="3"/>
       <c r="M4" s="3"/>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N4" s="3"/>
+      <c r="O4" s="3"/>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
         <v>3</v>
       </c>
@@ -11841,8 +11231,10 @@
       <c r="K5" s="3"/>
       <c r="L5" s="3"/>
       <c r="M5" s="3"/>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N5" s="3"/>
+      <c r="O5" s="3"/>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
         <v>4</v>
       </c>
@@ -11858,8 +11250,10 @@
       <c r="K6" s="3"/>
       <c r="L6" s="3"/>
       <c r="M6" s="3"/>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N6" s="3"/>
+      <c r="O6" s="3"/>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A7" s="3">
         <v>5</v>
       </c>
@@ -11875,8 +11269,10 @@
       <c r="K7" s="3"/>
       <c r="L7" s="3"/>
       <c r="M7" s="3"/>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N7" s="3"/>
+      <c r="O7" s="3"/>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
         <v>6</v>
       </c>
@@ -11892,8 +11288,10 @@
       <c r="K8" s="3"/>
       <c r="L8" s="3"/>
       <c r="M8" s="3"/>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N8" s="3"/>
+      <c r="O8" s="3"/>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
         <v>7</v>
       </c>
@@ -11909,8 +11307,10 @@
       <c r="K9" s="3"/>
       <c r="L9" s="3"/>
       <c r="M9" s="3"/>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N9" s="3"/>
+      <c r="O9" s="3"/>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
         <v>8</v>
       </c>
@@ -11926,8 +11326,10 @@
       <c r="K10" s="3"/>
       <c r="L10" s="3"/>
       <c r="M10" s="3"/>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N10" s="3"/>
+      <c r="O10" s="3"/>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>9</v>
       </c>
@@ -11943,8 +11345,10 @@
       <c r="K11" s="3"/>
       <c r="L11" s="3"/>
       <c r="M11" s="3"/>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N11" s="3"/>
+      <c r="O11" s="3"/>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>10</v>
       </c>
@@ -11960,196 +11364,30 @@
       <c r="K12" s="3"/>
       <c r="L12" s="3"/>
       <c r="M12" s="3"/>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A13" s="3">
-        <v>11</v>
-      </c>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
-      <c r="J13" s="3"/>
-      <c r="K13" s="3"/>
-      <c r="L13" s="3"/>
-      <c r="M13" s="3"/>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A14" s="3">
-        <v>12</v>
-      </c>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
-      <c r="J14" s="3"/>
-      <c r="K14" s="3"/>
-      <c r="L14" s="3"/>
-      <c r="M14" s="3"/>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A15" s="3">
-        <v>13</v>
-      </c>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
-      <c r="I15" s="3"/>
-      <c r="J15" s="3"/>
-      <c r="K15" s="3"/>
-      <c r="L15" s="3"/>
-      <c r="M15" s="3"/>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A16" s="3">
-        <v>14</v>
-      </c>
-      <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
-      <c r="F16" s="3"/>
-      <c r="G16" s="3"/>
-      <c r="H16" s="3"/>
-      <c r="I16" s="3"/>
-      <c r="J16" s="3"/>
-      <c r="K16" s="3"/>
-      <c r="L16" s="3"/>
-      <c r="M16" s="3"/>
-    </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A17" s="3">
-        <v>15</v>
-      </c>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
-      <c r="G17" s="3"/>
-      <c r="H17" s="3"/>
-      <c r="I17" s="3"/>
-      <c r="J17" s="3"/>
-      <c r="K17" s="3"/>
-      <c r="L17" s="3"/>
-      <c r="M17" s="3"/>
-    </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A18" s="3">
-        <v>16</v>
-      </c>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-      <c r="F18" s="3"/>
-      <c r="G18" s="3"/>
-      <c r="H18" s="3"/>
-      <c r="I18" s="3"/>
-      <c r="J18" s="3"/>
-      <c r="K18" s="3"/>
-      <c r="L18" s="3"/>
-      <c r="M18" s="3"/>
-    </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A19" s="3">
-        <v>17</v>
-      </c>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
-      <c r="I19" s="3"/>
-      <c r="J19" s="3"/>
-      <c r="K19" s="3"/>
-      <c r="L19" s="3"/>
-      <c r="M19" s="3"/>
-      <c r="O19" s="46"/>
-      <c r="P19" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A20" s="3">
-        <v>18</v>
-      </c>
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
-      <c r="F20" s="3"/>
-      <c r="G20" s="3"/>
-      <c r="H20" s="3"/>
-      <c r="I20" s="3"/>
-      <c r="J20" s="3"/>
-      <c r="K20" s="3"/>
-      <c r="L20" s="3"/>
-      <c r="M20" s="3"/>
-      <c r="O20" s="31"/>
-      <c r="P20" s="9" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A21" s="3">
-        <v>19</v>
-      </c>
-      <c r="B21" s="3"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
-      <c r="E21" s="3"/>
-      <c r="F21" s="3"/>
-      <c r="G21" s="3"/>
-      <c r="H21" s="3"/>
-      <c r="I21" s="3"/>
-      <c r="J21" s="3"/>
-      <c r="K21" s="3"/>
-      <c r="L21" s="3"/>
-      <c r="M21" s="3"/>
-      <c r="O21" s="34"/>
-      <c r="P21" s="9" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A22" s="3">
-        <v>20</v>
-      </c>
-      <c r="B22" s="3"/>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
-      <c r="E22" s="3"/>
-      <c r="F22" s="3"/>
-      <c r="G22" s="3"/>
-      <c r="H22" s="3"/>
-      <c r="I22" s="3"/>
-      <c r="J22" s="3"/>
-      <c r="K22" s="3"/>
-      <c r="L22" s="3"/>
-      <c r="M22" s="3"/>
-    </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="I24" s="9"/>
-      <c r="J24" s="9"/>
-    </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="I25" s="9"/>
-      <c r="J25" s="9"/>
+      <c r="N12" s="3"/>
+      <c r="O12" s="3"/>
+      <c r="Q12" s="45"/>
+      <c r="R12" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="Q13" s="31"/>
+      <c r="R13" s="9" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="I14" s="9"/>
+      <c r="J14" s="9"/>
+      <c r="Q14" s="34"/>
+      <c r="R14" s="9" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="I15" s="9"/>
+      <c r="J15" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -12171,34 +11409,34 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="B2" s="58" t="s">
+      <c r="B2" s="57" t="s">
         <v>138</v>
       </c>
-      <c r="C2" s="58"/>
-      <c r="E2" s="54" t="s">
+      <c r="C2" s="57"/>
+      <c r="E2" s="53" t="s">
         <v>133</v>
       </c>
-      <c r="F2" s="54"/>
-      <c r="H2" s="54" t="s">
+      <c r="F2" s="53"/>
+      <c r="H2" s="53" t="s">
         <v>134</v>
       </c>
-      <c r="I2" s="54"/>
-      <c r="K2" s="54" t="s">
+      <c r="I2" s="53"/>
+      <c r="K2" s="53" t="s">
         <v>135</v>
       </c>
-      <c r="L2" s="54"/>
-      <c r="N2" s="54" t="s">
+      <c r="L2" s="53"/>
+      <c r="N2" s="53" t="s">
         <v>136</v>
       </c>
-      <c r="O2" s="54"/>
-      <c r="Q2" s="54" t="s">
+      <c r="O2" s="53"/>
+      <c r="Q2" s="53" t="s">
         <v>137</v>
       </c>
-      <c r="R2" s="54"/>
+      <c r="R2" s="53"/>
     </row>
     <row r="3" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="B3" s="58"/>
-      <c r="C3" s="58"/>
+      <c r="B3" s="57"/>
+      <c r="C3" s="57"/>
       <c r="E3" s="37" t="s">
         <v>95</v>
       </c>
@@ -12565,34 +11803,34 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="B2" s="59" t="s">
+      <c r="B2" s="58" t="s">
         <v>140</v>
       </c>
-      <c r="C2" s="59"/>
-      <c r="E2" s="55" t="s">
+      <c r="C2" s="58"/>
+      <c r="E2" s="54" t="s">
         <v>139</v>
       </c>
-      <c r="F2" s="55"/>
-      <c r="H2" s="55" t="s">
+      <c r="F2" s="54"/>
+      <c r="H2" s="54" t="s">
         <v>141</v>
       </c>
-      <c r="I2" s="55"/>
-      <c r="K2" s="55" t="s">
+      <c r="I2" s="54"/>
+      <c r="K2" s="54" t="s">
         <v>142</v>
       </c>
-      <c r="L2" s="55"/>
-      <c r="N2" s="55" t="s">
+      <c r="L2" s="54"/>
+      <c r="N2" s="54" t="s">
         <v>143</v>
       </c>
-      <c r="O2" s="55"/>
-      <c r="Q2" s="55" t="s">
+      <c r="O2" s="54"/>
+      <c r="Q2" s="54" t="s">
         <v>144</v>
       </c>
-      <c r="R2" s="55"/>
+      <c r="R2" s="54"/>
     </row>
     <row r="3" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="B3" s="59"/>
-      <c r="C3" s="59"/>
+      <c r="B3" s="58"/>
+      <c r="C3" s="58"/>
       <c r="E3" s="39" t="s">
         <v>95</v>
       </c>
@@ -13030,36 +12268,36 @@
       <c r="Q6" s="1"/>
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="C7" s="48" t="s">
+      <c r="C7" s="47" t="s">
         <v>57</v>
       </c>
-      <c r="D7" s="48"/>
-      <c r="E7" s="48"/>
-      <c r="F7" s="48"/>
-      <c r="G7" s="48"/>
-      <c r="H7" s="48"/>
-      <c r="I7" s="48"/>
-      <c r="J7" s="48"/>
+      <c r="D7" s="47"/>
+      <c r="E7" s="47"/>
+      <c r="F7" s="47"/>
+      <c r="G7" s="47"/>
+      <c r="H7" s="47"/>
+      <c r="I7" s="47"/>
+      <c r="J7" s="47"/>
       <c r="K7" s="1"/>
-      <c r="L7" s="48" t="s">
+      <c r="L7" s="47" t="s">
         <v>58</v>
       </c>
-      <c r="M7" s="48"/>
-      <c r="N7" s="48"/>
-      <c r="O7" s="48"/>
-      <c r="P7" s="48"/>
-      <c r="Q7" s="48"/>
-      <c r="R7" s="48" t="s">
+      <c r="M7" s="47"/>
+      <c r="N7" s="47"/>
+      <c r="O7" s="47"/>
+      <c r="P7" s="47"/>
+      <c r="Q7" s="47"/>
+      <c r="R7" s="47" t="s">
         <v>93</v>
       </c>
-      <c r="S7" s="48"/>
-      <c r="T7" s="48"/>
-      <c r="U7" s="48"/>
-      <c r="V7" s="48"/>
-      <c r="W7" s="48" t="s">
+      <c r="S7" s="47"/>
+      <c r="T7" s="47"/>
+      <c r="U7" s="47"/>
+      <c r="V7" s="47"/>
+      <c r="W7" s="47" t="s">
         <v>100</v>
       </c>
-      <c r="X7" s="48"/>
+      <c r="X7" s="47"/>
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A8" s="20" t="s">
@@ -13917,74 +13155,74 @@
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="49" t="s">
+      <c r="A4" s="50" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="49"/>
-      <c r="D4" s="49" t="s">
+      <c r="B4" s="50"/>
+      <c r="D4" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="49"/>
-      <c r="G4" s="49" t="s">
+      <c r="E4" s="50"/>
+      <c r="G4" s="50" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="49"/>
-      <c r="J4" s="49" t="s">
+      <c r="H4" s="50"/>
+      <c r="J4" s="50" t="s">
         <v>7</v>
       </c>
-      <c r="K4" s="49"/>
-      <c r="M4" s="49" t="s">
+      <c r="K4" s="50"/>
+      <c r="M4" s="50" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="49"/>
-      <c r="P4" s="49" t="s">
+      <c r="N4" s="50"/>
+      <c r="P4" s="50" t="s">
         <v>9</v>
       </c>
-      <c r="Q4" s="49"/>
+      <c r="Q4" s="50"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="49" t="s">
+      <c r="S4" s="50" t="s">
         <v>10</v>
       </c>
-      <c r="T4" s="49"/>
+      <c r="T4" s="50"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="49" t="s">
+      <c r="V4" s="50" t="s">
         <v>11</v>
       </c>
-      <c r="W4" s="49"/>
+      <c r="W4" s="50"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="49" t="s">
+      <c r="Y4" s="50" t="s">
         <v>12</v>
       </c>
-      <c r="Z4" s="49"/>
+      <c r="Z4" s="50"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="49" t="s">
+      <c r="AB4" s="50" t="s">
         <v>13</v>
       </c>
-      <c r="AC4" s="49"/>
-      <c r="AE4" s="49" t="s">
+      <c r="AC4" s="50"/>
+      <c r="AE4" s="50" t="s">
         <v>114</v>
       </c>
-      <c r="AF4" s="49"/>
+      <c r="AF4" s="50"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="49" t="s">
+      <c r="AH4" s="50" t="s">
         <v>115</v>
       </c>
-      <c r="AI4" s="49"/>
+      <c r="AI4" s="50"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="49" t="s">
+      <c r="AK4" s="50" t="s">
         <v>116</v>
       </c>
-      <c r="AL4" s="49"/>
+      <c r="AL4" s="50"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="49" t="s">
+      <c r="AN4" s="50" t="s">
         <v>117</v>
       </c>
-      <c r="AO4" s="49"/>
+      <c r="AO4" s="50"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="49" t="s">
+      <c r="AQ4" s="50" t="s">
         <v>118</v>
       </c>
-      <c r="AR4" s="49"/>
+      <c r="AR4" s="50"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="41" t="s">
@@ -14087,89 +13325,89 @@
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="50" t="str">
+      <c r="A6" s="48" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="B6" s="51"/>
-      <c r="D6" s="50" t="str">
+      <c r="B6" s="49"/>
+      <c r="D6" s="48" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="E6" s="51"/>
-      <c r="G6" s="50" t="str">
+      <c r="E6" s="49"/>
+      <c r="G6" s="48" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="H6" s="51"/>
-      <c r="J6" s="50" t="str">
+      <c r="H6" s="49"/>
+      <c r="J6" s="48" t="str">
         <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="K6" s="51"/>
-      <c r="M6" s="50" t="str">
+      <c r="K6" s="49"/>
+      <c r="M6" s="48" t="str">
         <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="N6" s="51"/>
-      <c r="P6" s="50" t="str">
+      <c r="N6" s="49"/>
+      <c r="P6" s="48" t="str">
         <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Q6" s="51"/>
+      <c r="Q6" s="49"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="50" t="str">
+      <c r="S6" s="48" t="str">
         <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="T6" s="51"/>
+      <c r="T6" s="49"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="50" t="str">
+      <c r="V6" s="48" t="str">
         <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="W6" s="51"/>
+      <c r="W6" s="49"/>
       <c r="X6" s="1"/>
-      <c r="Y6" s="50" t="str">
+      <c r="Y6" s="48" t="str">
         <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Z6" s="51"/>
+      <c r="Z6" s="49"/>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="50" t="str">
+      <c r="AB6" s="48" t="str">
         <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AC6" s="51"/>
-      <c r="AE6" s="50" t="str">
+      <c r="AC6" s="49"/>
+      <c r="AE6" s="48" t="str">
         <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AF6" s="51"/>
+      <c r="AF6" s="49"/>
       <c r="AG6" s="1"/>
-      <c r="AH6" s="50" t="str">
+      <c r="AH6" s="48" t="str">
         <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AI6" s="51"/>
+      <c r="AI6" s="49"/>
       <c r="AJ6" s="1"/>
-      <c r="AK6" s="50" t="str">
+      <c r="AK6" s="48" t="str">
         <f>_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AL6" s="51"/>
+      <c r="AL6" s="49"/>
       <c r="AM6" s="1"/>
-      <c r="AN6" s="50" t="str">
+      <c r="AN6" s="48" t="str">
         <f>_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AO6" s="51"/>
+      <c r="AO6" s="49"/>
       <c r="AP6" s="1"/>
-      <c r="AQ6" s="50" t="str">
+      <c r="AQ6" s="48" t="str">
         <f>_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AR6" s="51"/>
+      <c r="AR6" s="49"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -15073,36 +14311,36 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="V4:W4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AE4:AF4"/>
+    <mergeCell ref="AH4:AI4"/>
+    <mergeCell ref="AK4:AL4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="AQ4:AR4"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
     <mergeCell ref="AE6:AF6"/>
     <mergeCell ref="AH6:AI6"/>
     <mergeCell ref="AK6:AL6"/>
     <mergeCell ref="AN6:AO6"/>
     <mergeCell ref="AQ6:AR6"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="AE4:AF4"/>
-    <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="AK4:AL4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="AQ4:AR4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="S4:T4"/>
-    <mergeCell ref="V4:W4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -15136,78 +14374,78 @@
   <sheetData>
     <row r="2" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A2" s="27" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="49" t="s">
+      <c r="A4" s="50" t="s">
         <v>153</v>
       </c>
-      <c r="B4" s="49"/>
-      <c r="D4" s="49" t="s">
+      <c r="B4" s="50"/>
+      <c r="D4" s="50" t="s">
         <v>154</v>
       </c>
-      <c r="E4" s="49"/>
-      <c r="G4" s="49" t="s">
+      <c r="E4" s="50"/>
+      <c r="G4" s="50" t="s">
         <v>155</v>
       </c>
-      <c r="H4" s="49"/>
-      <c r="J4" s="49" t="s">
+      <c r="H4" s="50"/>
+      <c r="J4" s="50" t="s">
         <v>156</v>
       </c>
-      <c r="K4" s="49"/>
-      <c r="M4" s="49" t="s">
+      <c r="K4" s="50"/>
+      <c r="M4" s="50" t="s">
         <v>157</v>
       </c>
-      <c r="N4" s="49"/>
-      <c r="P4" s="49" t="s">
+      <c r="N4" s="50"/>
+      <c r="P4" s="50" t="s">
         <v>158</v>
       </c>
-      <c r="Q4" s="49"/>
+      <c r="Q4" s="50"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="49" t="s">
+      <c r="S4" s="50" t="s">
         <v>159</v>
       </c>
-      <c r="T4" s="49"/>
+      <c r="T4" s="50"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="49" t="s">
+      <c r="V4" s="50" t="s">
         <v>160</v>
       </c>
-      <c r="W4" s="49"/>
+      <c r="W4" s="50"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="49" t="s">
+      <c r="Y4" s="50" t="s">
         <v>161</v>
       </c>
-      <c r="Z4" s="49"/>
+      <c r="Z4" s="50"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="49" t="s">
+      <c r="AB4" s="50" t="s">
         <v>162</v>
       </c>
-      <c r="AC4" s="49"/>
-      <c r="AE4" s="49" t="s">
+      <c r="AC4" s="50"/>
+      <c r="AE4" s="50" t="s">
         <v>163</v>
       </c>
-      <c r="AF4" s="49"/>
+      <c r="AF4" s="50"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="49" t="s">
+      <c r="AH4" s="50" t="s">
         <v>164</v>
       </c>
-      <c r="AI4" s="49"/>
+      <c r="AI4" s="50"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="49" t="s">
+      <c r="AK4" s="50" t="s">
         <v>165</v>
       </c>
-      <c r="AL4" s="49"/>
+      <c r="AL4" s="50"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="49" t="s">
+      <c r="AN4" s="50" t="s">
         <v>166</v>
       </c>
-      <c r="AO4" s="49"/>
+      <c r="AO4" s="50"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="49" t="s">
+      <c r="AQ4" s="50" t="s">
         <v>167</v>
       </c>
-      <c r="AR4" s="49"/>
+      <c r="AR4" s="50"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="43" t="s">
@@ -15310,89 +14548,89 @@
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="52" t="str">
+      <c r="A6" s="51" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="B6" s="53"/>
-      <c r="D6" s="52" t="str">
+      <c r="B6" s="52"/>
+      <c r="D6" s="51" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="E6" s="53"/>
-      <c r="G6" s="52" t="str">
+      <c r="E6" s="52"/>
+      <c r="G6" s="51" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="H6" s="53"/>
-      <c r="J6" s="52" t="str">
+      <c r="H6" s="52"/>
+      <c r="J6" s="51" t="str">
         <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="K6" s="53"/>
-      <c r="M6" s="52" t="str">
+      <c r="K6" s="52"/>
+      <c r="M6" s="51" t="str">
         <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="N6" s="53"/>
-      <c r="P6" s="52" t="str">
+      <c r="N6" s="52"/>
+      <c r="P6" s="51" t="str">
         <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Q6" s="53"/>
+      <c r="Q6" s="52"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="52" t="str">
+      <c r="S6" s="51" t="str">
         <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="T6" s="53"/>
+      <c r="T6" s="52"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="52" t="str">
+      <c r="V6" s="51" t="str">
         <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="W6" s="53"/>
+      <c r="W6" s="52"/>
       <c r="X6" s="1"/>
-      <c r="Y6" s="52" t="str">
+      <c r="Y6" s="51" t="str">
         <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Z6" s="53"/>
+      <c r="Z6" s="52"/>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="52" t="str">
+      <c r="AB6" s="51" t="str">
         <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AC6" s="53"/>
-      <c r="AE6" s="52" t="str">
+      <c r="AC6" s="52"/>
+      <c r="AE6" s="51" t="str">
         <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AF6" s="53"/>
+      <c r="AF6" s="52"/>
       <c r="AG6" s="1"/>
-      <c r="AH6" s="52" t="str">
+      <c r="AH6" s="51" t="str">
         <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AI6" s="53"/>
+      <c r="AI6" s="52"/>
       <c r="AJ6" s="1"/>
-      <c r="AK6" s="52" t="str">
+      <c r="AK6" s="51" t="str">
         <f>_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AL6" s="53"/>
+      <c r="AL6" s="52"/>
       <c r="AM6" s="1"/>
-      <c r="AN6" s="52" t="str">
+      <c r="AN6" s="51" t="str">
         <f>_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AO6" s="53"/>
+      <c r="AO6" s="52"/>
       <c r="AP6" s="1"/>
-      <c r="AQ6" s="52" t="str">
+      <c r="AQ6" s="51" t="str">
         <f>_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AR6" s="53"/>
+      <c r="AR6" s="52"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -16296,14 +15534,12 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AQ6:AR6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AE6:AF6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="AK6:AL6"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
     <mergeCell ref="AK4:AL4"/>
     <mergeCell ref="AN4:AO4"/>
     <mergeCell ref="AQ4:AR4"/>
@@ -16320,12 +15556,14 @@
     <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="AE4:AF4"/>
     <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AQ6:AR6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AE6:AF6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="AK6:AL6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -16341,14 +15579,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="54" t="s">
+      <c r="A2" s="53" t="s">
         <v>84</v>
       </c>
-      <c r="B2" s="54"/>
-      <c r="D2" s="55" t="s">
+      <c r="B2" s="53"/>
+      <c r="D2" s="54" t="s">
         <v>82</v>
       </c>
-      <c r="E2" s="55"/>
+      <c r="E2" s="54"/>
       <c r="G2" s="24" t="s">
         <v>83</v>
       </c>
@@ -16887,36 +16125,36 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B2" s="56" t="s">
+      <c r="B2" s="55" t="s">
         <v>127</v>
       </c>
-      <c r="C2" s="56"/>
-      <c r="D2" s="56"/>
-      <c r="F2" s="56" t="s">
+      <c r="C2" s="55"/>
+      <c r="D2" s="55"/>
+      <c r="F2" s="55" t="s">
         <v>128</v>
       </c>
-      <c r="G2" s="56"/>
-      <c r="H2" s="56"/>
-      <c r="J2" s="56" t="s">
+      <c r="G2" s="55"/>
+      <c r="H2" s="55"/>
+      <c r="J2" s="55" t="s">
         <v>129</v>
       </c>
-      <c r="K2" s="56"/>
-      <c r="L2" s="56"/>
-      <c r="N2" s="56" t="s">
+      <c r="K2" s="55"/>
+      <c r="L2" s="55"/>
+      <c r="N2" s="55" t="s">
         <v>130</v>
       </c>
-      <c r="O2" s="56"/>
-      <c r="P2" s="56"/>
-      <c r="R2" s="56" t="s">
+      <c r="O2" s="55"/>
+      <c r="P2" s="55"/>
+      <c r="R2" s="55" t="s">
         <v>131</v>
       </c>
-      <c r="S2" s="56"/>
-      <c r="T2" s="56"/>
-      <c r="V2" s="56" t="s">
+      <c r="S2" s="55"/>
+      <c r="T2" s="55"/>
+      <c r="V2" s="55" t="s">
         <v>132</v>
       </c>
-      <c r="W2" s="56"/>
-      <c r="X2" s="56"/>
+      <c r="W2" s="55"/>
+      <c r="X2" s="55"/>
     </row>
     <row r="3" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">

</xml_diff>

<commit_message>
implement V_cap and M_cap structural capacity checks for LEM piles
Add optional Vcap and Mcap columns to the piles sheet. When provided,
the per-pile force is capped at the lesser of soil capacity, shear
capacity (V_cap), and moment capacity (M_cap / L_m) before entering
the equilibrium equations. L_m is computed exactly from the Ito &
Matsui pressure centroid, or defaults to depth/3 for user-specified H.

Also refactors Ito & Matsui, rapid drawdown, and no-solution summary
printing from main_lem.py into reusable functions in xslope/summary.py.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/inputs/input_template_v10.xlsx
+++ b/docs/inputs/input_template_v10.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BBAABD4-E426-8F49-8470-E5780033835C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{504986E3-C218-E64B-BA82-5C812B1ECEB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="24480" yWindow="2380" windowWidth="42700" windowHeight="22800" activeTab="11" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="24880" yWindow="1600" windowWidth="42700" windowHeight="22800" activeTab="11" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -1193,7 +1193,12 @@
     <xf numFmtId="0" fontId="16" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1233,12 +1238,7 @@
     <xf numFmtId="0" fontId="1" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -9261,13 +9261,13 @@
       <xdr:col>11</xdr:col>
       <xdr:colOff>553357</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>99787</xdr:rowOff>
+      <xdr:rowOff>99788</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
       <xdr:colOff>780143</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>54428</xdr:rowOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>181429</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -9282,8 +9282,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9180286" y="498930"/>
-          <a:ext cx="4354286" cy="2748641"/>
+          <a:off x="9180286" y="498931"/>
+          <a:ext cx="4354286" cy="1877784"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -9331,20 +9331,14 @@
           </a:r>
         </a:p>
         <a:p>
-          <a:endParaRPr lang="en-US" sz="1100" baseline="0"/>
-        </a:p>
-        <a:p>
           <a:r>
             <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
             <a:t>Tmax</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1100" baseline="0"/>
-            <a:t> = maximum tensile strength of reinforcement material. </a:t>
+            <a:t> = maximum tensile strength (per unit width) of reinforcement material. </a:t>
           </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1100" baseline="0"/>
         </a:p>
         <a:p>
           <a:r>
@@ -9353,11 +9347,8 @@
           </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1100" baseline="0"/>
-            <a:t> = residual strenth of reinfocement material.</a:t>
+            <a:t> = residual strenth (per unit width) of reinfocement material.</a:t>
           </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1100" baseline="0"/>
         </a:p>
         <a:p>
           <a:r>
@@ -9372,9 +9363,6 @@
             <a:rPr lang="en-US" sz="1100" baseline="0"/>
             <a:t> length or length required to generate full frictional resistance on end corresponding to point 1.</a:t>
           </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1100" baseline="0"/>
         </a:p>
         <a:p>
           <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
@@ -9408,20 +9396,31 @@
           </a:r>
         </a:p>
         <a:p>
-          <a:endParaRPr lang="en-US" sz="1100" baseline="0"/>
-        </a:p>
-        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
           <a:r>
             <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
             <a:t>E</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1100" baseline="0"/>
-            <a:t> = modulus of elasticity of reinforcement material</a:t>
+            <a:t> = Young's modulus of reinforcement material (force/length^2)</a:t>
           </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1100" baseline="0"/>
         </a:p>
         <a:p>
           <a:r>
@@ -9430,7 +9429,7 @@
           </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1100" baseline="0"/>
-            <a:t> = cross-sectional area (per unit width) of reinforcement material </a:t>
+            <a:t> = cross-sectional area (per unit width) of reinforcement material.</a:t>
           </a:r>
           <a:endParaRPr lang="en-US" sz="1100"/>
         </a:p>
@@ -9451,8 +9450,8 @@
       <xdr:rowOff>18144</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>163285</xdr:colOff>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>680357</xdr:colOff>
       <xdr:row>10</xdr:row>
       <xdr:rowOff>63500</xdr:rowOff>
     </xdr:to>
@@ -9470,7 +9469,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="12273642" y="217715"/>
-          <a:ext cx="4826000" cy="1841499"/>
+          <a:ext cx="3156858" cy="1841499"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -10110,11 +10109,11 @@
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B7" s="46" t="s">
+      <c r="B7" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="C7" s="46"/>
-      <c r="D7" s="46"/>
+      <c r="C7" s="47"/>
+      <c r="D7" s="47"/>
       <c r="F7" s="15" t="s">
         <v>15</v>
       </c>
@@ -10273,36 +10272,36 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B2" s="56" t="s">
+      <c r="B2" s="57" t="s">
         <v>145</v>
       </c>
-      <c r="C2" s="56"/>
-      <c r="D2" s="56"/>
-      <c r="F2" s="56" t="s">
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="F2" s="57" t="s">
         <v>146</v>
       </c>
-      <c r="G2" s="56"/>
-      <c r="H2" s="56"/>
-      <c r="J2" s="56" t="s">
+      <c r="G2" s="57"/>
+      <c r="H2" s="57"/>
+      <c r="J2" s="57" t="s">
         <v>147</v>
       </c>
-      <c r="K2" s="56"/>
-      <c r="L2" s="56"/>
-      <c r="N2" s="56" t="s">
+      <c r="K2" s="57"/>
+      <c r="L2" s="57"/>
+      <c r="N2" s="57" t="s">
         <v>148</v>
       </c>
-      <c r="O2" s="56"/>
-      <c r="P2" s="56"/>
-      <c r="R2" s="56" t="s">
+      <c r="O2" s="57"/>
+      <c r="P2" s="57"/>
+      <c r="R2" s="57" t="s">
         <v>149</v>
       </c>
-      <c r="S2" s="56"/>
-      <c r="T2" s="56"/>
-      <c r="V2" s="56" t="s">
+      <c r="S2" s="57"/>
+      <c r="T2" s="57"/>
+      <c r="V2" s="57" t="s">
         <v>150</v>
       </c>
-      <c r="W2" s="56"/>
-      <c r="X2" s="56"/>
+      <c r="W2" s="57"/>
+      <c r="X2" s="57"/>
     </row>
     <row r="3" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">
@@ -10760,9 +10759,10 @@
   <cols>
     <col min="1" max="1" width="4.83203125" style="1" customWidth="1"/>
     <col min="2" max="11" width="10.83203125" style="1"/>
+    <col min="12" max="12" width="7.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
         <v>25</v>
       </c>
@@ -10797,7 +10797,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>1</v>
       </c>
@@ -10812,7 +10812,7 @@
       <c r="J3" s="3"/>
       <c r="K3" s="3"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>2</v>
       </c>
@@ -10827,7 +10827,7 @@
       <c r="J4" s="3"/>
       <c r="K4" s="3"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
         <v>3</v>
       </c>
@@ -10842,7 +10842,7 @@
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
         <v>4</v>
       </c>
@@ -10857,7 +10857,7 @@
       <c r="J6" s="3"/>
       <c r="K6" s="3"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A7" s="3">
         <v>5</v>
       </c>
@@ -10872,7 +10872,7 @@
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
         <v>6</v>
       </c>
@@ -10887,7 +10887,7 @@
       <c r="J8" s="3"/>
       <c r="K8" s="3"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
         <v>7</v>
       </c>
@@ -10902,7 +10902,7 @@
       <c r="J9" s="3"/>
       <c r="K9" s="3"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
         <v>8</v>
       </c>
@@ -10917,7 +10917,7 @@
       <c r="J10" s="3"/>
       <c r="K10" s="3"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>9</v>
       </c>
@@ -10932,7 +10932,7 @@
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>10</v>
       </c>
@@ -10947,7 +10947,7 @@
       <c r="J12" s="3"/>
       <c r="K12" s="3"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <v>11</v>
       </c>
@@ -10962,7 +10962,7 @@
       <c r="J13" s="3"/>
       <c r="K13" s="3"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <v>12</v>
       </c>
@@ -10976,8 +10976,12 @@
       <c r="I14" s="3"/>
       <c r="J14" s="3"/>
       <c r="K14" s="3"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="M14" s="31"/>
+      <c r="N14" s="9" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
         <v>13</v>
       </c>
@@ -10991,8 +10995,12 @@
       <c r="I15" s="3"/>
       <c r="J15" s="3"/>
       <c r="K15" s="3"/>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="M15" s="34"/>
+      <c r="N15" s="9" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>14</v>
       </c>
@@ -11007,7 +11015,7 @@
       <c r="J16" s="3"/>
       <c r="K16" s="3"/>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
         <v>15</v>
       </c>
@@ -11022,7 +11030,7 @@
       <c r="J17" s="3"/>
       <c r="K17" s="3"/>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
         <v>16</v>
       </c>
@@ -11037,7 +11045,7 @@
       <c r="J18" s="3"/>
       <c r="K18" s="3"/>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
         <v>17</v>
       </c>
@@ -11051,12 +11059,8 @@
       <c r="I19" s="3"/>
       <c r="J19" s="3"/>
       <c r="K19" s="3"/>
-      <c r="M19" s="31"/>
-      <c r="N19" s="9" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
         <v>18</v>
       </c>
@@ -11070,12 +11074,8 @@
       <c r="I20" s="3"/>
       <c r="J20" s="3"/>
       <c r="K20" s="3"/>
-      <c r="M20" s="34"/>
-      <c r="N20" s="9" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" s="3">
         <v>19</v>
       </c>
@@ -11090,7 +11090,7 @@
       <c r="J21" s="3"/>
       <c r="K21" s="3"/>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" s="3">
         <v>20</v>
       </c>
@@ -11105,11 +11105,11 @@
       <c r="J22" s="3"/>
       <c r="K22" s="3"/>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="H24" s="9"/>
       <c r="I24" s="9"/>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="H25" s="9"/>
       <c r="I25" s="9"/>
     </row>
@@ -11149,10 +11149,10 @@
       <c r="F2" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="G2" s="59" t="s">
+      <c r="G2" s="45" t="s">
         <v>168</v>
       </c>
-      <c r="H2" s="59" t="s">
+      <c r="H2" s="45" t="s">
         <v>176</v>
       </c>
       <c r="I2" s="32" t="s">
@@ -11170,10 +11170,10 @@
       <c r="M2" s="33" t="s">
         <v>107</v>
       </c>
-      <c r="N2" s="60" t="s">
+      <c r="N2" s="46" t="s">
         <v>173</v>
       </c>
-      <c r="O2" s="60" t="s">
+      <c r="O2" s="46" t="s">
         <v>174</v>
       </c>
     </row>
@@ -11366,7 +11366,7 @@
       <c r="M12" s="3"/>
       <c r="N12" s="3"/>
       <c r="O12" s="3"/>
-      <c r="Q12" s="45"/>
+      <c r="Q12" s="60"/>
       <c r="R12" t="s">
         <v>177</v>
       </c>
@@ -11409,34 +11409,34 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="B2" s="57" t="s">
+      <c r="B2" s="58" t="s">
         <v>138</v>
       </c>
-      <c r="C2" s="57"/>
-      <c r="E2" s="53" t="s">
+      <c r="C2" s="58"/>
+      <c r="E2" s="54" t="s">
         <v>133</v>
       </c>
-      <c r="F2" s="53"/>
-      <c r="H2" s="53" t="s">
+      <c r="F2" s="54"/>
+      <c r="H2" s="54" t="s">
         <v>134</v>
       </c>
-      <c r="I2" s="53"/>
-      <c r="K2" s="53" t="s">
+      <c r="I2" s="54"/>
+      <c r="K2" s="54" t="s">
         <v>135</v>
       </c>
-      <c r="L2" s="53"/>
-      <c r="N2" s="53" t="s">
+      <c r="L2" s="54"/>
+      <c r="N2" s="54" t="s">
         <v>136</v>
       </c>
-      <c r="O2" s="53"/>
-      <c r="Q2" s="53" t="s">
+      <c r="O2" s="54"/>
+      <c r="Q2" s="54" t="s">
         <v>137</v>
       </c>
-      <c r="R2" s="53"/>
+      <c r="R2" s="54"/>
     </row>
     <row r="3" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="B3" s="57"/>
-      <c r="C3" s="57"/>
+      <c r="B3" s="58"/>
+      <c r="C3" s="58"/>
       <c r="E3" s="37" t="s">
         <v>95</v>
       </c>
@@ -11803,34 +11803,34 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="B2" s="58" t="s">
+      <c r="B2" s="59" t="s">
         <v>140</v>
       </c>
-      <c r="C2" s="58"/>
-      <c r="E2" s="54" t="s">
+      <c r="C2" s="59"/>
+      <c r="E2" s="55" t="s">
         <v>139</v>
       </c>
-      <c r="F2" s="54"/>
-      <c r="H2" s="54" t="s">
+      <c r="F2" s="55"/>
+      <c r="H2" s="55" t="s">
         <v>141</v>
       </c>
-      <c r="I2" s="54"/>
-      <c r="K2" s="54" t="s">
+      <c r="I2" s="55"/>
+      <c r="K2" s="55" t="s">
         <v>142</v>
       </c>
-      <c r="L2" s="54"/>
-      <c r="N2" s="54" t="s">
+      <c r="L2" s="55"/>
+      <c r="N2" s="55" t="s">
         <v>143</v>
       </c>
-      <c r="O2" s="54"/>
-      <c r="Q2" s="54" t="s">
+      <c r="O2" s="55"/>
+      <c r="Q2" s="55" t="s">
         <v>144</v>
       </c>
-      <c r="R2" s="54"/>
+      <c r="R2" s="55"/>
     </row>
     <row r="3" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="B3" s="58"/>
-      <c r="C3" s="58"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="59"/>
       <c r="E3" s="39" t="s">
         <v>95</v>
       </c>
@@ -12268,36 +12268,36 @@
       <c r="Q6" s="1"/>
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="C7" s="47" t="s">
+      <c r="C7" s="48" t="s">
         <v>57</v>
       </c>
-      <c r="D7" s="47"/>
-      <c r="E7" s="47"/>
-      <c r="F7" s="47"/>
-      <c r="G7" s="47"/>
-      <c r="H7" s="47"/>
-      <c r="I7" s="47"/>
-      <c r="J7" s="47"/>
+      <c r="D7" s="48"/>
+      <c r="E7" s="48"/>
+      <c r="F7" s="48"/>
+      <c r="G7" s="48"/>
+      <c r="H7" s="48"/>
+      <c r="I7" s="48"/>
+      <c r="J7" s="48"/>
       <c r="K7" s="1"/>
-      <c r="L7" s="47" t="s">
+      <c r="L7" s="48" t="s">
         <v>58</v>
       </c>
-      <c r="M7" s="47"/>
-      <c r="N7" s="47"/>
-      <c r="O7" s="47"/>
-      <c r="P7" s="47"/>
-      <c r="Q7" s="47"/>
-      <c r="R7" s="47" t="s">
+      <c r="M7" s="48"/>
+      <c r="N7" s="48"/>
+      <c r="O7" s="48"/>
+      <c r="P7" s="48"/>
+      <c r="Q7" s="48"/>
+      <c r="R7" s="48" t="s">
         <v>93</v>
       </c>
-      <c r="S7" s="47"/>
-      <c r="T7" s="47"/>
-      <c r="U7" s="47"/>
-      <c r="V7" s="47"/>
-      <c r="W7" s="47" t="s">
+      <c r="S7" s="48"/>
+      <c r="T7" s="48"/>
+      <c r="U7" s="48"/>
+      <c r="V7" s="48"/>
+      <c r="W7" s="48" t="s">
         <v>100</v>
       </c>
-      <c r="X7" s="47"/>
+      <c r="X7" s="48"/>
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A8" s="20" t="s">
@@ -13155,74 +13155,74 @@
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="50" t="s">
+      <c r="A4" s="51" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="50"/>
-      <c r="D4" s="50" t="s">
+      <c r="B4" s="51"/>
+      <c r="D4" s="51" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="50"/>
-      <c r="G4" s="50" t="s">
+      <c r="E4" s="51"/>
+      <c r="G4" s="51" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="50"/>
-      <c r="J4" s="50" t="s">
+      <c r="H4" s="51"/>
+      <c r="J4" s="51" t="s">
         <v>7</v>
       </c>
-      <c r="K4" s="50"/>
-      <c r="M4" s="50" t="s">
+      <c r="K4" s="51"/>
+      <c r="M4" s="51" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="50"/>
-      <c r="P4" s="50" t="s">
+      <c r="N4" s="51"/>
+      <c r="P4" s="51" t="s">
         <v>9</v>
       </c>
-      <c r="Q4" s="50"/>
+      <c r="Q4" s="51"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="50" t="s">
+      <c r="S4" s="51" t="s">
         <v>10</v>
       </c>
-      <c r="T4" s="50"/>
+      <c r="T4" s="51"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="50" t="s">
+      <c r="V4" s="51" t="s">
         <v>11</v>
       </c>
-      <c r="W4" s="50"/>
+      <c r="W4" s="51"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="50" t="s">
+      <c r="Y4" s="51" t="s">
         <v>12</v>
       </c>
-      <c r="Z4" s="50"/>
+      <c r="Z4" s="51"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="50" t="s">
+      <c r="AB4" s="51" t="s">
         <v>13</v>
       </c>
-      <c r="AC4" s="50"/>
-      <c r="AE4" s="50" t="s">
+      <c r="AC4" s="51"/>
+      <c r="AE4" s="51" t="s">
         <v>114</v>
       </c>
-      <c r="AF4" s="50"/>
+      <c r="AF4" s="51"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="50" t="s">
+      <c r="AH4" s="51" t="s">
         <v>115</v>
       </c>
-      <c r="AI4" s="50"/>
+      <c r="AI4" s="51"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="50" t="s">
+      <c r="AK4" s="51" t="s">
         <v>116</v>
       </c>
-      <c r="AL4" s="50"/>
+      <c r="AL4" s="51"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="50" t="s">
+      <c r="AN4" s="51" t="s">
         <v>117</v>
       </c>
-      <c r="AO4" s="50"/>
+      <c r="AO4" s="51"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="50" t="s">
+      <c r="AQ4" s="51" t="s">
         <v>118</v>
       </c>
-      <c r="AR4" s="50"/>
+      <c r="AR4" s="51"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="41" t="s">
@@ -13325,89 +13325,89 @@
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="48" t="str">
+      <c r="A6" s="49" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="B6" s="49"/>
-      <c r="D6" s="48" t="str">
+      <c r="B6" s="50"/>
+      <c r="D6" s="49" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="E6" s="49"/>
-      <c r="G6" s="48" t="str">
+      <c r="E6" s="50"/>
+      <c r="G6" s="49" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="H6" s="49"/>
-      <c r="J6" s="48" t="str">
+      <c r="H6" s="50"/>
+      <c r="J6" s="49" t="str">
         <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="K6" s="49"/>
-      <c r="M6" s="48" t="str">
+      <c r="K6" s="50"/>
+      <c r="M6" s="49" t="str">
         <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="N6" s="49"/>
-      <c r="P6" s="48" t="str">
+      <c r="N6" s="50"/>
+      <c r="P6" s="49" t="str">
         <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Q6" s="49"/>
+      <c r="Q6" s="50"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="48" t="str">
+      <c r="S6" s="49" t="str">
         <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="T6" s="49"/>
+      <c r="T6" s="50"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="48" t="str">
+      <c r="V6" s="49" t="str">
         <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="W6" s="49"/>
+      <c r="W6" s="50"/>
       <c r="X6" s="1"/>
-      <c r="Y6" s="48" t="str">
+      <c r="Y6" s="49" t="str">
         <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Z6" s="49"/>
+      <c r="Z6" s="50"/>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="48" t="str">
+      <c r="AB6" s="49" t="str">
         <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AC6" s="49"/>
-      <c r="AE6" s="48" t="str">
+      <c r="AC6" s="50"/>
+      <c r="AE6" s="49" t="str">
         <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AF6" s="49"/>
+      <c r="AF6" s="50"/>
       <c r="AG6" s="1"/>
-      <c r="AH6" s="48" t="str">
+      <c r="AH6" s="49" t="str">
         <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AI6" s="49"/>
+      <c r="AI6" s="50"/>
       <c r="AJ6" s="1"/>
-      <c r="AK6" s="48" t="str">
+      <c r="AK6" s="49" t="str">
         <f>_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AL6" s="49"/>
+      <c r="AL6" s="50"/>
       <c r="AM6" s="1"/>
-      <c r="AN6" s="48" t="str">
+      <c r="AN6" s="49" t="str">
         <f>_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AO6" s="49"/>
+      <c r="AO6" s="50"/>
       <c r="AP6" s="1"/>
-      <c r="AQ6" s="48" t="str">
+      <c r="AQ6" s="49" t="str">
         <f>_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AR6" s="49"/>
+      <c r="AR6" s="50"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -14378,74 +14378,74 @@
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="50" t="s">
+      <c r="A4" s="51" t="s">
         <v>153</v>
       </c>
-      <c r="B4" s="50"/>
-      <c r="D4" s="50" t="s">
+      <c r="B4" s="51"/>
+      <c r="D4" s="51" t="s">
         <v>154</v>
       </c>
-      <c r="E4" s="50"/>
-      <c r="G4" s="50" t="s">
+      <c r="E4" s="51"/>
+      <c r="G4" s="51" t="s">
         <v>155</v>
       </c>
-      <c r="H4" s="50"/>
-      <c r="J4" s="50" t="s">
+      <c r="H4" s="51"/>
+      <c r="J4" s="51" t="s">
         <v>156</v>
       </c>
-      <c r="K4" s="50"/>
-      <c r="M4" s="50" t="s">
+      <c r="K4" s="51"/>
+      <c r="M4" s="51" t="s">
         <v>157</v>
       </c>
-      <c r="N4" s="50"/>
-      <c r="P4" s="50" t="s">
+      <c r="N4" s="51"/>
+      <c r="P4" s="51" t="s">
         <v>158</v>
       </c>
-      <c r="Q4" s="50"/>
+      <c r="Q4" s="51"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="50" t="s">
+      <c r="S4" s="51" t="s">
         <v>159</v>
       </c>
-      <c r="T4" s="50"/>
+      <c r="T4" s="51"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="50" t="s">
+      <c r="V4" s="51" t="s">
         <v>160</v>
       </c>
-      <c r="W4" s="50"/>
+      <c r="W4" s="51"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="50" t="s">
+      <c r="Y4" s="51" t="s">
         <v>161</v>
       </c>
-      <c r="Z4" s="50"/>
+      <c r="Z4" s="51"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="50" t="s">
+      <c r="AB4" s="51" t="s">
         <v>162</v>
       </c>
-      <c r="AC4" s="50"/>
-      <c r="AE4" s="50" t="s">
+      <c r="AC4" s="51"/>
+      <c r="AE4" s="51" t="s">
         <v>163</v>
       </c>
-      <c r="AF4" s="50"/>
+      <c r="AF4" s="51"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="50" t="s">
+      <c r="AH4" s="51" t="s">
         <v>164</v>
       </c>
-      <c r="AI4" s="50"/>
+      <c r="AI4" s="51"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="50" t="s">
+      <c r="AK4" s="51" t="s">
         <v>165</v>
       </c>
-      <c r="AL4" s="50"/>
+      <c r="AL4" s="51"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="50" t="s">
+      <c r="AN4" s="51" t="s">
         <v>166</v>
       </c>
-      <c r="AO4" s="50"/>
+      <c r="AO4" s="51"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="50" t="s">
+      <c r="AQ4" s="51" t="s">
         <v>167</v>
       </c>
-      <c r="AR4" s="50"/>
+      <c r="AR4" s="51"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="43" t="s">
@@ -14548,89 +14548,89 @@
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="51" t="str">
+      <c r="A6" s="52" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="B6" s="52"/>
-      <c r="D6" s="51" t="str">
+      <c r="B6" s="53"/>
+      <c r="D6" s="52" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="E6" s="52"/>
-      <c r="G6" s="51" t="str">
+      <c r="E6" s="53"/>
+      <c r="G6" s="52" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="H6" s="52"/>
-      <c r="J6" s="51" t="str">
+      <c r="H6" s="53"/>
+      <c r="J6" s="52" t="str">
         <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="K6" s="52"/>
-      <c r="M6" s="51" t="str">
+      <c r="K6" s="53"/>
+      <c r="M6" s="52" t="str">
         <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="N6" s="52"/>
-      <c r="P6" s="51" t="str">
+      <c r="N6" s="53"/>
+      <c r="P6" s="52" t="str">
         <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Q6" s="52"/>
+      <c r="Q6" s="53"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="51" t="str">
+      <c r="S6" s="52" t="str">
         <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="T6" s="52"/>
+      <c r="T6" s="53"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="51" t="str">
+      <c r="V6" s="52" t="str">
         <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="W6" s="52"/>
+      <c r="W6" s="53"/>
       <c r="X6" s="1"/>
-      <c r="Y6" s="51" t="str">
+      <c r="Y6" s="52" t="str">
         <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Z6" s="52"/>
+      <c r="Z6" s="53"/>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="51" t="str">
+      <c r="AB6" s="52" t="str">
         <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AC6" s="52"/>
-      <c r="AE6" s="51" t="str">
+      <c r="AC6" s="53"/>
+      <c r="AE6" s="52" t="str">
         <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AF6" s="52"/>
+      <c r="AF6" s="53"/>
       <c r="AG6" s="1"/>
-      <c r="AH6" s="51" t="str">
+      <c r="AH6" s="52" t="str">
         <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AI6" s="52"/>
+      <c r="AI6" s="53"/>
       <c r="AJ6" s="1"/>
-      <c r="AK6" s="51" t="str">
+      <c r="AK6" s="52" t="str">
         <f>_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AL6" s="52"/>
+      <c r="AL6" s="53"/>
       <c r="AM6" s="1"/>
-      <c r="AN6" s="51" t="str">
+      <c r="AN6" s="52" t="str">
         <f>_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AO6" s="52"/>
+      <c r="AO6" s="53"/>
       <c r="AP6" s="1"/>
-      <c r="AQ6" s="51" t="str">
+      <c r="AQ6" s="52" t="str">
         <f>_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AR6" s="52"/>
+      <c r="AR6" s="53"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -15579,14 +15579,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="53" t="s">
+      <c r="A2" s="54" t="s">
         <v>84</v>
       </c>
-      <c r="B2" s="53"/>
-      <c r="D2" s="54" t="s">
+      <c r="B2" s="54"/>
+      <c r="D2" s="55" t="s">
         <v>82</v>
       </c>
-      <c r="E2" s="54"/>
+      <c r="E2" s="55"/>
       <c r="G2" s="24" t="s">
         <v>83</v>
       </c>
@@ -16125,36 +16125,36 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B2" s="55" t="s">
+      <c r="B2" s="56" t="s">
         <v>127</v>
       </c>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="F2" s="55" t="s">
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="F2" s="56" t="s">
         <v>128</v>
       </c>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
-      <c r="J2" s="55" t="s">
+      <c r="G2" s="56"/>
+      <c r="H2" s="56"/>
+      <c r="J2" s="56" t="s">
         <v>129</v>
       </c>
-      <c r="K2" s="55"/>
-      <c r="L2" s="55"/>
-      <c r="N2" s="55" t="s">
+      <c r="K2" s="56"/>
+      <c r="L2" s="56"/>
+      <c r="N2" s="56" t="s">
         <v>130</v>
       </c>
-      <c r="O2" s="55"/>
-      <c r="P2" s="55"/>
-      <c r="R2" s="55" t="s">
+      <c r="O2" s="56"/>
+      <c r="P2" s="56"/>
+      <c r="R2" s="56" t="s">
         <v>131</v>
       </c>
-      <c r="S2" s="55"/>
-      <c r="T2" s="55"/>
-      <c r="V2" s="55" t="s">
+      <c r="S2" s="56"/>
+      <c r="T2" s="56"/>
+      <c r="V2" s="56" t="s">
         <v>132</v>
       </c>
-      <c r="W2" s="55"/>
-      <c r="X2" s="55"/>
+      <c r="W2" s="56"/>
+      <c r="X2" s="56"/>
     </row>
     <row r="3" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">

</xml_diff>